<commit_message>
updated stage gating problem
</commit_message>
<xml_diff>
--- a/Logic/Milestone_Register_Oct1.xlsx
+++ b/Logic/Milestone_Register_Oct1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gosciminski/Documents/GitHub/M-GRAT/Logic/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93AE4F4D-824D-BE44-8988-68231BDC7586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71C76DFB-8D16-954D-9C56-35509C078FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19780" yWindow="-21000" windowWidth="34580" windowHeight="20200" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19780" yWindow="-21000" windowWidth="34580" windowHeight="20200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Added comment in Excel to fix FSM1 recommendations
</commit_message>
<xml_diff>
--- a/Logic/Milestone_Register_Oct1.xlsx
+++ b/Logic/Milestone_Register_Oct1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gosciminski/Documents/GitHub/M-GRAT/Logic/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyletran/Documents/GitHub/M-GRAT/Logic/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71C76DFB-8D16-954D-9C56-35509C078FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED9AB61-D493-4848-BB05-8D029E19C239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19780" yWindow="-21000" windowWidth="34580" windowHeight="20200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-50560" yWindow="-2020" windowWidth="45080" windowHeight="21680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -24,10 +24,37 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Milestone Actions'!$A$1:$D$117</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Milestone Register'!$A$1:$N$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Milestone Register'!$A$1:$N$62</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={4AA0F2E5-F17B-1341-9B6E-AF8BB0E2DA95}</author>
+    <author>tc={1C4FD9E7-5BC6-254F-9926-B56171CF8847}</author>
+  </authors>
+  <commentList>
+    <comment ref="M15" authorId="0" shapeId="0" xr:uid="{4AA0F2E5-F17B-1341-9B6E-AF8BB0E2DA95}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This needs to be something else</t>
+      </text>
+    </comment>
+    <comment ref="M46" authorId="1" shapeId="0" xr:uid="{1C4FD9E7-5BC6-254F-9926-B56171CF8847}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This needs to be something else</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3929,7 +3956,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4020,6 +4047,12 @@
       <b/>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -4621,6 +4654,12 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Kyle Tran" id="{8F59DB08-9212-9B41-BB4D-CC2F3AA04612}" userId="S::Kyle.Tran@ibm.com::1e0920c3-21ee-4bb1-8116-08da48d74603" providerId="AD"/>
+</personList>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4904,6 +4943,17 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="M15" dT="2026-10-15T09:58:54.91" personId="{8F59DB08-9212-9B41-BB4D-CC2F3AA04612}" id="{4AA0F2E5-F17B-1341-9B6E-AF8BB0E2DA95}">
+    <text>This needs to be something else</text>
+  </threadedComment>
+  <threadedComment ref="M46" dT="2026-10-15T09:59:22.26" personId="{8F59DB08-9212-9B41-BB4D-CC2F3AA04612}" id="{1C4FD9E7-5BC6-254F-9926-B56171CF8847}">
+    <text>This needs to be something else</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D29"/>
@@ -5112,7 +5162,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:Q62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.1640625" defaultRowHeight="129" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -5237,7 +5288,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>116</v>
       </c>
@@ -5290,7 +5341,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>128</v>
       </c>
@@ -5343,7 +5394,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>142</v>
       </c>
@@ -5396,7 +5447,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>154</v>
       </c>
@@ -5502,7 +5553,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>175</v>
       </c>
@@ -5555,7 +5606,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>185</v>
       </c>
@@ -5608,7 +5659,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>196</v>
       </c>
@@ -5661,7 +5712,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>207</v>
       </c>
@@ -5714,7 +5765,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>218</v>
       </c>
@@ -5767,7 +5818,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>231</v>
       </c>
@@ -5820,7 +5871,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>244</v>
       </c>
@@ -5926,7 +5977,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>268</v>
       </c>
@@ -5979,7 +6030,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>279</v>
       </c>
@@ -6032,7 +6083,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>291</v>
       </c>
@@ -6138,7 +6189,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="20" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>313</v>
       </c>
@@ -6191,7 +6242,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="21" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>325</v>
       </c>
@@ -6244,7 +6295,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>336</v>
       </c>
@@ -6297,7 +6348,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="23" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>348</v>
       </c>
@@ -6403,7 +6454,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="25" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>370</v>
       </c>
@@ -6456,7 +6507,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="26" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>382</v>
       </c>
@@ -6509,7 +6560,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="27" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>394</v>
       </c>
@@ -6562,7 +6613,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="28" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>406</v>
       </c>
@@ -6668,7 +6719,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="30" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>429</v>
       </c>
@@ -6721,7 +6772,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="31" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>440</v>
       </c>
@@ -6774,7 +6825,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="32" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>452</v>
       </c>
@@ -6827,7 +6878,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="33" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>462</v>
       </c>
@@ -6880,7 +6931,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="34" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>473</v>
       </c>
@@ -6933,7 +6984,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="35" spans="1:17" s="14" customFormat="1" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:17" s="14" customFormat="1" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="14" t="s">
         <v>484</v>
       </c>
@@ -6986,7 +7037,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="36" spans="1:17" ht="144" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:17" ht="144" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>496</v>
       </c>
@@ -7039,7 +7090,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="37" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>507</v>
       </c>
@@ -7092,7 +7143,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="38" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>519</v>
       </c>
@@ -7145,7 +7196,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="39" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>531</v>
       </c>
@@ -7198,7 +7249,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="40" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>543</v>
       </c>
@@ -7251,7 +7302,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="41" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>556</v>
       </c>
@@ -7304,7 +7355,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="42" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>567</v>
       </c>
@@ -7357,7 +7408,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="43" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>579</v>
       </c>
@@ -7410,7 +7461,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="44" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>589</v>
       </c>
@@ -7463,7 +7514,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="45" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>600</v>
       </c>
@@ -7569,7 +7620,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="47" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>622</v>
       </c>
@@ -7622,7 +7673,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="48" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>632</v>
       </c>
@@ -7675,7 +7726,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="49" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>644</v>
       </c>
@@ -7728,7 +7779,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="50" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>656</v>
       </c>
@@ -7781,7 +7832,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="51" spans="1:17" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:17" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>668</v>
       </c>
@@ -7834,7 +7885,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="52" spans="1:17" s="14" customFormat="1" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:17" s="14" customFormat="1" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>679</v>
       </c>
@@ -7887,7 +7938,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="53" spans="1:17" s="14" customFormat="1" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:17" s="14" customFormat="1" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="14" t="s">
         <v>690</v>
       </c>
@@ -7993,7 +8044,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="55" spans="1:17" s="14" customFormat="1" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:17" s="14" customFormat="1" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="14" t="s">
         <v>713</v>
       </c>
@@ -8043,7 +8094,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="56" spans="1:17" s="14" customFormat="1" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:17" s="14" customFormat="1" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="14" t="s">
         <v>723</v>
       </c>
@@ -8093,7 +8144,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="57" spans="1:17" s="14" customFormat="1" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:17" s="14" customFormat="1" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="14" t="s">
         <v>733</v>
       </c>
@@ -8143,7 +8194,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="58" spans="1:17" s="14" customFormat="1" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:17" s="14" customFormat="1" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="14" t="s">
         <v>744</v>
       </c>
@@ -8193,7 +8244,7 @@
         <v>754</v>
       </c>
     </row>
-    <row r="59" spans="1:17" s="14" customFormat="1" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:17" s="14" customFormat="1" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="14" t="s">
         <v>755</v>
       </c>
@@ -8243,7 +8294,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="60" spans="1:17" s="14" customFormat="1" ht="129" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:17" s="14" customFormat="1" ht="129" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
         <v>766</v>
       </c>
@@ -8293,7 +8344,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="61" spans="1:17" s="14" customFormat="1" ht="144" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:17" s="14" customFormat="1" ht="144" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="14" t="s">
         <v>778</v>
       </c>
@@ -8343,7 +8394,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="62" spans="1:17" ht="144" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:17" ht="144" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="14" t="s">
         <v>790</v>
       </c>
@@ -8394,8 +8445,15 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N44" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:N62" xr:uid="{00000000-0009-0000-0000-000001000000}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="FSM1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat(report): show stage "Are you ready" text; update FSM readiness wording
- Milestone Register: rewrite FSM Stage 2-5 "Are you ready" statements
- build_report_data.py: read the "Are you ready" column into readinessText
  (it previously read a nonexistent "Milestones" column, so all 10 stages
  were null)
- report.js: render "Are you ready?" on the target-stage expansion card
- docs/index.html: refresh embedded Opportunity paths data (page + PDF)
- Regenerate data/*.js and the self-serve bundles (root and docs/)
- wiki/Changelog.md: add week of 23-29 Oct entry
</commit_message>
<xml_diff>
--- a/Logic/Milestone_Register_Oct1.xlsx
+++ b/Logic/Milestone_Register_Oct1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyletran/Documents/GitHub/M-GRAT/Logic/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED9AB61-D493-4848-BB05-8D029E19C239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2666C395-EAFE-4740-B49A-64C5D1493643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-50560" yWindow="-2020" windowWidth="45080" windowHeight="21680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1724" uniqueCount="1141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1724" uniqueCount="1142">
   <si>
     <t>Capability Pillar / Domain</t>
   </si>
@@ -3940,23 +3940,26 @@
     <t>Labour records, craft classifications, calendar/shift definitions, and basic job plan templates are established. Work orders carry scheduled dates.</t>
   </si>
   <si>
-    <t>Work orders carry scheduled dates and a forward planning horizon is established (weekly to monthly). A centralized scheduler or dispatcher role is active in Assignment Manager, workforce availability is enriched with exceptions, and job plans gain materials, tools, and classifications. HSE, Inspections, and Inventory enter as parallel capability layers.</t>
-  </si>
-  <si>
-    <t>Forward planning extends to rolling windows with predecessor and hierarchy constraints. System-suggested dispatch based on effective availability is active. Job plans are scoped to asset classes, include hierarchies and predecessors, and link to asset data. Inspection results feed condition data and inventory is planned against work requirements.</t>
-  </si>
-  <si>
-    <t>The Optimizer runs automatically via cron-based scheduling. Assignments are system-generated from constraints, skills, and optimized availability. Planning, Scheduling, and Dispatch dashboards are live with cost, resource, and compliance views. Condition-based inspection and optimized inventory management are active.</t>
-  </si>
-  <si>
     <t>Are you ready</t>
+  </si>
+  <si>
+    <t>Centralized schedule coordination and field dispatch — single-pane visibility across labor and crew capacity, extended planning horizons, and mobile work execution that eliminates paper delays.</t>
+  </si>
+  <si>
+    <t>Optimized crew productivity and work preparation — enriching job plans with planned materials and tools, sequencing work by dependencies, and routing technicians by geographic proximity.</t>
+  </si>
+  <si>
+    <t>Automated schedule optimization and exception handling — constraint-based algorithms match technicians by skill and location, inject emergency break-in work, and integrate storeroom inventory at the point of work.</t>
+  </si>
+  <si>
+    <t>Achieved autonomous, end-to-end field workforce execution — automated cron-based optimization, GenAI point-of-work troubleshooting, and real-time field actuals driving continuous schedule refinement.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4047,12 +4050,6 @@
       <b/>
       <sz val="10"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -10180,7 +10177,7 @@
         <v>1121</v>
       </c>
       <c r="I1" s="25" t="s">
-        <v>1140</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="96" customHeight="1" x14ac:dyDescent="0.2">
@@ -10238,7 +10235,7 @@
         <v>1123</v>
       </c>
       <c r="I3" s="44" t="s">
-        <v>1137</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="96" customHeight="1" x14ac:dyDescent="0.2">
@@ -10267,7 +10264,7 @@
         <v>1124</v>
       </c>
       <c r="I4" s="44" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="96" customHeight="1" x14ac:dyDescent="0.2">
@@ -10296,7 +10293,7 @@
         <v>1125</v>
       </c>
       <c r="I5" s="44" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
@@ -10325,7 +10322,7 @@
         <v>1126</v>
       </c>
       <c r="I6" s="44" t="s">
-        <v>993</v>
+        <v>1141</v>
       </c>
     </row>
   </sheetData>
@@ -10375,7 +10372,7 @@
         <v>1121</v>
       </c>
       <c r="I1" s="25" t="s">
-        <v>1140</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="190" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>